<commit_message>
Added write of run update files.
</commit_message>
<xml_diff>
--- a/analysis/resources/plate_templates/APLATE.v2.0.0.xlsx
+++ b/analysis/resources/plate_templates/APLATE.v2.0.0.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/analysis/resources/plate_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F53A1F7-A062-C843-A4D5-3D04437C50D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1EECB59-6C3E-524C-BBCD-410D7CBD55E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51460" yWindow="120" windowWidth="27600" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="6" r:id="rId1"/>
     <sheet name="Plate" sheetId="3" r:id="rId2"/>
-    <sheet name="Volumes" sheetId="8" r:id="rId3"/>
+    <sheet name="Volume Overrides" sheetId="8" r:id="rId3"/>
     <sheet name="Comments" sheetId="4" r:id="rId4"/>
     <sheet name="Run Setup" sheetId="2" r:id="rId5"/>
     <sheet name="Lists" sheetId="5" r:id="rId6"/>
@@ -456,12 +456,6 @@
     <t>Genomic Element</t>
   </si>
   <si>
-    <t>Control 1 Calculated Copies Per Reaction</t>
-  </si>
-  <si>
-    <t>Control 2 Calculated Copies Per Reaction</t>
-  </si>
-  <si>
     <t>Fluorophore</t>
   </si>
   <si>
@@ -481,9 +475,6 @@
   </si>
   <si>
     <t>Target</t>
-  </si>
-  <si>
-    <t>Calculated Copies Per Reaction</t>
   </si>
   <si>
     <t>Categories</t>
@@ -540,9 +531,6 @@
     <t>Method Lot ID</t>
   </si>
   <si>
-    <t>Input mL</t>
-  </si>
-  <si>
     <t>Target Category</t>
   </si>
   <si>
@@ -555,10 +543,22 @@
     <t>PCR NC</t>
   </si>
   <si>
-    <t>* Amount of extraction included in each reaction. Can be overriden for single wells in the "Volumes" sheet.</t>
+    <t>APX</t>
   </si>
   <si>
-    <t>APX</t>
+    <t>* Amount of extraction included in each reaction. Can be overriden for single wells in the "Volume Overrides" sheet.</t>
+  </si>
+  <si>
+    <t>Input uL</t>
+  </si>
+  <si>
+    <t>Calculated Copies Per uL Reaction</t>
+  </si>
+  <si>
+    <t>Control 1 Calculated Copies Per uL Reaction</t>
+  </si>
+  <si>
+    <t>Control 2 Calculated Copies Per uL Reaction</t>
   </si>
 </sst>
 </file>
@@ -1707,7 +1707,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="69" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C6" s="69"/>
       <c r="D6" s="63"/>
@@ -1736,13 +1736,13 @@
     </row>
     <row r="7" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="67" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B7" s="71">
-        <v>5.0000000000000001E-3</v>
+        <v>5</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D7" s="63"/>
       <c r="E7" s="63"/>
@@ -1832,7 +1832,7 @@
     </row>
     <row r="10" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="69" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B10" s="69" t="s">
         <v>117</v>
@@ -1864,10 +1864,10 @@
     </row>
     <row r="11" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="71" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B11" s="71" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C11" s="65"/>
       <c r="D11" s="63"/>
@@ -1896,7 +1896,7 @@
     </row>
     <row r="12" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="69" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B12" s="69" t="s">
         <v>81</v>
@@ -1928,7 +1928,7 @@
     </row>
     <row r="13" spans="1:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="72" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B13" s="72"/>
       <c r="C13" s="73"/>
@@ -1958,7 +1958,7 @@
     </row>
     <row r="14" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="74" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B14" s="74" t="s">
         <v>63</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="15" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="80" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B15" s="80" t="s">
         <v>84</v>
@@ -2021,16 +2021,16 @@
     </row>
     <row r="16" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="87" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B16" s="88" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C16" s="81"/>
     </row>
     <row r="17" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="80" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B17" s="80" t="s">
         <v>129</v>
@@ -2094,7 +2094,7 @@
     </row>
     <row r="19" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="80" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="B19" s="80"/>
       <c r="C19" s="65"/>
@@ -2176,7 +2176,7 @@
         <v>119</v>
       </c>
       <c r="B23" s="76" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C23" s="81"/>
       <c r="E23" s="63"/>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="24" spans="1:26" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="77" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="B24" s="77">
         <v>0</v>
@@ -2334,7 +2334,7 @@
         <v>120</v>
       </c>
       <c r="B28" s="79" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C28" s="65"/>
       <c r="D28" s="63"/>
@@ -2363,7 +2363,7 @@
     </row>
     <row r="29" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="79" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
       <c r="B29" s="79"/>
       <c r="C29" s="65"/>
@@ -2393,7 +2393,7 @@
     </row>
     <row r="30" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="85" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B30" s="85" t="s">
         <v>68</v>
@@ -2424,7 +2424,7 @@
     </row>
     <row r="31" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="80" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B31" s="80" t="s">
         <v>84</v>
@@ -2456,10 +2456,10 @@
     </row>
     <row r="32" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="87" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B32" s="88" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D32" s="63"/>
       <c r="E32" s="63"/>
@@ -2487,7 +2487,7 @@
     </row>
     <row r="33" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="80" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B33" s="80" t="s">
         <v>129</v>
@@ -2551,7 +2551,7 @@
     </row>
     <row r="35" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="80" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="B35" s="80"/>
       <c r="C35" s="63"/>
@@ -2677,7 +2677,7 @@
         <v>119</v>
       </c>
       <c r="B39" s="76" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D39" s="63"/>
       <c r="E39" s="63"/>
@@ -2705,7 +2705,7 @@
     </row>
     <row r="40" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="77" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="B40" s="77">
         <v>0</v>
@@ -2836,7 +2836,7 @@
         <v>120</v>
       </c>
       <c r="B44" s="79" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C44" s="63"/>
       <c r="D44" s="63"/>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="45" spans="1:26" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="79" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
       <c r="B45" s="79"/>
       <c r="C45" s="63"/>
@@ -2895,7 +2895,7 @@
     </row>
     <row r="46" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="85" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B46" s="85" t="s">
         <v>65</v>
@@ -2926,10 +2926,10 @@
     </row>
     <row r="47" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="80" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B47" s="80" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C47" s="63"/>
       <c r="D47" s="63"/>
@@ -2958,10 +2958,10 @@
     </row>
     <row r="48" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="87" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B48" s="88" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C48" s="63"/>
       <c r="D48" s="63"/>
@@ -2990,7 +2990,7 @@
     </row>
     <row r="49" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="80" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B49" s="80" t="s">
         <v>130</v>
@@ -3054,7 +3054,7 @@
     </row>
     <row r="51" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="80" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="B51" s="80">
         <v>0</v>
@@ -3182,7 +3182,7 @@
         <v>119</v>
       </c>
       <c r="B55" s="76" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D55" s="63"/>
       <c r="E55" s="63"/>
@@ -3210,7 +3210,7 @@
     </row>
     <row r="56" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="77" t="s">
-        <v>138</v>
+        <v>171</v>
       </c>
       <c r="B56" s="77">
         <v>0</v>
@@ -3362,7 +3362,7 @@
     </row>
     <row r="61" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="79" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
       <c r="B61" s="79"/>
       <c r="C61" s="63"/>
@@ -38841,10 +38841,10 @@
         <v>58</v>
       </c>
       <c r="C1" s="46" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E1" s="46" t="s">
         <v>106</v>
@@ -38903,7 +38903,7 @@
         <v>117</v>
       </c>
       <c r="K2" s="58" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L2" s="47" t="s">
         <v>81</v>
@@ -38920,7 +38920,7 @@
         <v>137</v>
       </c>
       <c r="D3" s="89" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E3" s="47" t="s">
         <v>95</v>
@@ -38958,7 +38958,7 @@
         <v>130</v>
       </c>
       <c r="D4" s="89" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E4" s="47" t="s">
         <v>96</v>
@@ -38979,7 +38979,7 @@
         <v>74</v>
       </c>
       <c r="K4" s="58" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="L4" s="48" t="s">
         <v>89</v>
@@ -39024,7 +39024,7 @@
         <v>133</v>
       </c>
       <c r="D6" s="90" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E6" s="51" t="s">
         <v>74</v>
@@ -39046,13 +39046,13 @@
     <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="48"/>
       <c r="B7" s="58" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C7" s="58" t="s">
         <v>134</v>
       </c>
       <c r="D7" s="90" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E7" s="48"/>
       <c r="F7" s="47" t="s">
@@ -39077,7 +39077,7 @@
         <v>135</v>
       </c>
       <c r="D8" s="90" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="E8" s="48"/>
       <c r="F8" s="47" t="s">
@@ -39097,13 +39097,13 @@
     <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="48"/>
       <c r="B9" s="86" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C9" s="51" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="90" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E9" s="48"/>
       <c r="F9" s="57" t="s">
@@ -39125,7 +39125,7 @@
       </c>
       <c r="C10" s="48"/>
       <c r="D10" s="90" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E10" s="48"/>
       <c r="F10" s="51" t="s">
@@ -39147,7 +39147,7 @@
       </c>
       <c r="C11" s="48"/>
       <c r="D11" s="90" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F11" s="48"/>
       <c r="G11" s="48"/>
@@ -39164,7 +39164,7 @@
       <c r="B12" s="48"/>
       <c r="C12" s="48"/>
       <c r="D12" s="90" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E12" s="48"/>
       <c r="F12" s="48"/>
@@ -39182,7 +39182,7 @@
       <c r="B13" s="48"/>
       <c r="C13" s="48"/>
       <c r="D13" s="90" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E13" s="48"/>
       <c r="F13" s="48"/>
@@ -39200,7 +39200,7 @@
       <c r="B14" s="48"/>
       <c r="C14" s="48"/>
       <c r="D14" s="90" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E14" s="48"/>
       <c r="F14" s="48"/>
@@ -39269,7 +39269,7 @@
     </row>
     <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D18" s="90" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="L18" s="48" t="s">
         <v>79</v>
@@ -39285,7 +39285,7 @@
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D20" s="86" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>